<commit_message>
feat: website inputs v1 — new OC members, cleaner photos, 26 answers
- Add Shivangi Sharma and Garvit Gosain to the organising committee
  (initials until their photos arrive)
- Crop the poster's navy/white border off every portrait
- Reword the Delhi weather paragraph; drop "A day, roughly" from Schedule
- Publish the settled answers: dates final, Asia Pacific eligibility,
  university-level sign-up, USD 630 fee and what it covers, scholarship,
  invited adjudicators, 8 prelims and motion timing, the break, buses,
  contact email, senior advisor surnames and bios
- Add the 19 regional advisors' records from the bid document
- Build log and open-decisions sheet cut from 26 open items to 16
- Keep the footer at the bottom on short pages

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/open-decisions.xlsx
+++ b/public/open-decisions.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -567,13 +567,17 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Confirm 27 June to 4 July 2027 is final, and not moving</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
+          <t>The cap on teams per university</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Depends on how many registrations come in; the constitution is being checked</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="9" t="n">
@@ -586,13 +590,13 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Which countries and regions are eligible</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr"/>
-      <c r="E7" s="10" t="inlineStr"/>
-      <c r="F7" s="10" t="inlineStr"/>
-      <c r="G7" s="10" t="inlineStr"/>
+          <t>The day registration opens and the day it closes</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="10" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="n">
@@ -600,18 +604,22 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Money</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>The cap on teams per university</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr"/>
-      <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="6" t="inlineStr"/>
-      <c r="G8" s="6" t="inlineStr"/>
+          <t>How people pay, and the payment deadlines</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>This decides which payment company we sign up with</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="9" t="n">
@@ -619,22 +627,18 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Money</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Whether a debater signs up for themselves, or their university signs up for its teams</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>This changes the shape of the registration form, so it is worth settling early</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr"/>
-      <c r="F9" s="10" t="inlineStr"/>
-      <c r="G9" s="10" t="inlineStr"/>
+          <t>Who sits on the Scholarship Board</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="n">
@@ -642,18 +646,22 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Judging</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>The day registration opens and the day it closes</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr"/>
-      <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="6" t="inlineStr"/>
+          <t>Confirm the judge rule is N−1</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>The site says it is expected, not settled</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="9" t="n">
@@ -661,18 +669,18 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Money</t>
+          <t>Rounds</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>The entry fee, and exactly what it covers</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr"/>
-      <c r="E11" s="10" t="inlineStr"/>
-      <c r="F11" s="10" t="inlineStr"/>
-      <c r="G11" s="10" t="inlineStr"/>
+          <t>How many teams break in Open, ESL and EFL</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="5" t="n">
@@ -680,18 +688,22 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Money</t>
+          <t>Rounds</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Whether accommodation at The Grand sits inside the fee or on top of it</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr"/>
-      <c r="E12" s="6" t="inlineStr"/>
-      <c r="F12" s="6" t="inlineStr"/>
-      <c r="G12" s="6" t="inlineStr"/>
+          <t>The day-by-day running order</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Which round falls on which day, socials, bus times</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="9" t="n">
@@ -699,22 +711,18 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Money</t>
+          <t>Rounds</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>How people pay: card, bank transfer or UPI</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>This decides which payment company we sign up with</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr"/>
-      <c r="F13" s="10" t="inlineStr"/>
-      <c r="G13" s="10" t="inlineStr"/>
+          <t>Whether the existing tab software stays, or is wired into this site</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="5" t="n">
@@ -722,18 +730,18 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Money</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>The scholarship route: who it is for, and what it covers</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr"/>
-      <c r="E14" s="6" t="inlineStr"/>
-      <c r="F14" s="6" t="inlineStr"/>
-      <c r="G14" s="6" t="inlineStr"/>
+          <t>Who sits on the equity team, and the confidential address to reach them</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="9" t="n">
@@ -741,18 +749,22 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Judging</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>How many judges a team must bring</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr"/>
-      <c r="E15" s="10" t="inlineStr"/>
-      <c r="F15" s="10" t="inlineStr"/>
-      <c r="G15" s="10" t="inlineStr"/>
+          <t>The equity policy, written out in full</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Published by the equity team with input from the adjudication core and Org Comm</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="5" t="n">
@@ -760,18 +772,18 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Judging</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Whether independent adjudicator applications are capped, and how they are assessed</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr"/>
-      <c r="E16" s="6" t="inlineStr"/>
-      <c r="F16" s="6" t="inlineStr"/>
-      <c r="G16" s="6" t="inlineStr"/>
+          <t>The participant handbook</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="9" t="n">
@@ -779,18 +791,22 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Rounds</t>
+          <t>Logistics</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>How many preliminary rounds, and how many motions go out in advance</t>
-        </is>
-      </c>
-      <c r="D17" s="12" t="inlineStr"/>
-      <c r="E17" s="10" t="inlineStr"/>
-      <c r="F17" s="10" t="inlineStr"/>
-      <c r="G17" s="10" t="inlineStr"/>
+          <t>When we can issue visa invitation letters</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Waiting on IIT Delhi to confirm its timelines and co-sign</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="5" t="n">
@@ -798,18 +814,22 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Rounds</t>
+          <t>Logistics</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>The break structure: Open, ESL, EFL, and how many teams in each</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr"/>
-      <c r="E18" s="6" t="inlineStr"/>
-      <c r="F18" s="6" t="inlineStr"/>
-      <c r="G18" s="6" t="inlineStr"/>
+          <t>A room-by-room access survey of the campus and the hotel</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Which rooms are step-free, where the accessible toilets are, the longest walk between rooms, ground-floor hotel rooms</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="9" t="n">
@@ -817,18 +837,22 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Rounds</t>
+          <t>Website</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>The day-by-day running order</t>
-        </is>
-      </c>
-      <c r="D19" s="12" t="inlineStr"/>
-      <c r="E19" s="10" t="inlineStr"/>
-      <c r="F19" s="10" t="inlineStr"/>
-      <c r="G19" s="10" t="inlineStr"/>
+          <t>A web address of our own</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>indiaaustrals2027.com, or close to it, is the preference</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="5" t="n">
@@ -836,18 +860,22 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Rounds</t>
+          <t>Website</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Whether the existing tab software stays, or is wired into this site</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr"/>
-      <c r="E20" s="6" t="inlineStr"/>
-      <c r="F20" s="6" t="inlineStr"/>
-      <c r="G20" s="6" t="inlineStr"/>
+          <t>How long we keep people's details after the tournament ends</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Previous organising committees are being asked what they did</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="9" t="n">
@@ -855,229 +883,33 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>People</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>Who sits on the equity team, and the confidential address to reach them</t>
-        </is>
-      </c>
-      <c r="D21" s="12" t="inlineStr"/>
-      <c r="E21" s="10" t="inlineStr"/>
-      <c r="F21" s="10" t="inlineStr"/>
-      <c r="G21" s="10" t="inlineStr"/>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>The equity policy, written out in full</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr"/>
-      <c r="E22" s="6" t="inlineStr"/>
-      <c r="F22" s="6" t="inlineStr"/>
-      <c r="G22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>The participant handbook, written out</t>
-        </is>
-      </c>
-      <c r="D23" s="12" t="inlineStr"/>
-      <c r="E23" s="10" t="inlineStr"/>
-      <c r="F23" s="10" t="inlineStr"/>
-      <c r="G23" s="10" t="inlineStr"/>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>Logistics</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>How teams get between The Grand and campus each morning, and who pays for it</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr"/>
-      <c r="E24" s="6" t="inlineStr"/>
-      <c r="F24" s="6" t="inlineStr"/>
-      <c r="G24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>Logistics</t>
-        </is>
-      </c>
-      <c r="C25" s="11" t="inlineStr">
-        <is>
-          <t>When we can issue visa invitation letters, and what they cover</t>
-        </is>
-      </c>
-      <c r="D25" s="12" t="inlineStr"/>
-      <c r="E25" s="10" t="inlineStr"/>
-      <c r="F25" s="10" t="inlineStr"/>
-      <c r="G25" s="10" t="inlineStr"/>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="5" t="n">
-        <v>21</v>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Logistics</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>A room-by-room access survey of the campus and the hotel</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>So we can say what is step-free instead of assuming</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr"/>
-      <c r="F26" s="6" t="inlineStr"/>
-      <c r="G26" s="6" t="inlineStr"/>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="B27" s="10" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>The email address the site should send from</t>
-        </is>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t>Confirmation emails need an address that is ours and that will not land in spam</t>
-        </is>
-      </c>
-      <c r="E27" s="10" t="inlineStr"/>
-      <c r="F27" s="10" t="inlineStr"/>
-      <c r="G27" s="10" t="inlineStr"/>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="5" t="n">
-        <v>23</v>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>A web address of our own to put the site on</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>It sits on a free address today, which works but does not read as ours</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr"/>
-      <c r="F28" s="6" t="inlineStr"/>
-      <c r="G28" s="6" t="inlineStr"/>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="inlineStr">
-        <is>
-          <t>How long we keep people's details after the tournament ends</t>
-        </is>
-      </c>
-      <c r="D29" s="12" t="inlineStr"/>
-      <c r="E29" s="10" t="inlineStr"/>
-      <c r="F29" s="10" t="inlineStr"/>
-      <c r="G29" s="10" t="inlineStr"/>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>People</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Surnames for Anjali and Kamal, our two senior advisors</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Their posters only carry first names</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr"/>
-      <c r="F30" s="6" t="inlineStr"/>
-      <c r="G30" s="6" t="inlineStr"/>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>People</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>Debating records for the twenty-one advisors</t>
-        </is>
-      </c>
-      <c r="D31" s="12" t="inlineStr">
-        <is>
-          <t>The posters carry their names and countries and nothing else</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="inlineStr"/>
-      <c r="F31" s="10" t="inlineStr"/>
-      <c r="G31" s="10" t="inlineStr"/>
-    </row>
+          <t>Photos of Shivangi Sharma and Garvit Gosain</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>They are on the site with their initials until then</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="10" t="n"/>
+    </row>
+    <row r="22" ht="30" customHeight="1"/>
+    <row r="23" ht="30" customHeight="1"/>
+    <row r="24" ht="30" customHeight="1"/>
+    <row r="25" ht="30" customHeight="1"/>
+    <row r="26" ht="30" customHeight="1"/>
+    <row r="27" ht="30" customHeight="1"/>
+    <row r="28" ht="30" customHeight="1"/>
+    <row r="29" ht="30" customHeight="1"/>
+    <row r="30" ht="30" customHeight="1"/>
+    <row r="31" ht="30" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:F3"/>

</xml_diff>

<commit_message>
content: apply team answers A-H, Delhi photo carousels, centred page rail
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/open-decisions.xlsx
+++ b/public/open-decisions.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -562,19 +562,15 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>The cap on teams per university</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Depends on how many registrations come in; the constitution is being checked</t>
-        </is>
-      </c>
+          <t>Who sits on the equity team, and the confidential address to reach them</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
       <c r="G6" s="6" t="n"/>
@@ -585,321 +581,59 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>The day registration opens and the day it closes</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="n"/>
+          <t>The equity policy, written out in full</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Published by the equity team with input from the adjudication core and Org Comm</t>
+        </is>
+      </c>
       <c r="E7" s="10" t="n"/>
       <c r="F7" s="10" t="n"/>
       <c r="G7" s="10" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Money</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>How people pay, and the payment deadlines</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>This decides which payment company we sign up with</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Photos of Shivangi Sharma and Garvit Gosain</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>They are on the site with their initials until then</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="10" t="n"/>
     </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>Money</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>Who sits on the Scholarship Board</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Judging</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Confirm the judge rule is N−1</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>The site says it is expected, not settled</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Rounds</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>How many teams break in Open, ESL and EFL</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Rounds</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>The day-by-day running order</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Which round falls on which day, socials, bus times</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Rounds</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>Whether the existing tab software stays, or is wired into this site</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Who sits on the equity team, and the confidential address to reach them</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="n"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>The equity policy, written out in full</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>Published by the equity team with input from the adjudication core and Org Comm</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>The participant handbook</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n"/>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Logistics</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>When we can issue visa invitation letters</t>
-        </is>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>Waiting on IIT Delhi to confirm its timelines and co-sign</t>
-        </is>
-      </c>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Logistics</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>A room-by-room access survey of the campus and the hotel</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Which rooms are step-free, where the accessible toilets are, the longest walk between rooms, ground-floor hotel rooms</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="6" t="n"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="9" t="n">
-        <v>14</v>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
-          <t>A web address of our own</t>
-        </is>
-      </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>indiaaustrals2027.com, or close to it, is the preference</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>How long we keep people's details after the tournament ends</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Previous organising committees are being asked what they did</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>People</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="inlineStr">
-        <is>
-          <t>Photos of Shivangi Sharma and Garvit Gosain</t>
-        </is>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>They are on the site with their initials until then</t>
-        </is>
-      </c>
-      <c r="E21" s="10" t="n"/>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="n"/>
-    </row>
+    <row r="9" ht="30" customHeight="1"/>
+    <row r="10" ht="30" customHeight="1"/>
+    <row r="11" ht="30" customHeight="1"/>
+    <row r="12" ht="30" customHeight="1"/>
+    <row r="13" ht="30" customHeight="1"/>
+    <row r="14" ht="30" customHeight="1"/>
+    <row r="15" ht="30" customHeight="1"/>
+    <row r="16" ht="30" customHeight="1"/>
+    <row r="17" ht="30" customHeight="1"/>
+    <row r="18" ht="30" customHeight="1"/>
+    <row r="19" ht="30" customHeight="1"/>
+    <row r="20" ht="30" customHeight="1"/>
+    <row r="21" ht="30" customHeight="1"/>
     <row r="22" ht="30" customHeight="1"/>
     <row r="23" ht="30" customHeight="1"/>
     <row r="24" ht="30" customHeight="1"/>

</xml_diff>

<commit_message>
content: plain-language rewrite of all site text, fact fixes, Shivangi's photo
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/open-decisions.xlsx
+++ b/public/open-decisions.xlsx
@@ -567,7 +567,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Who sits on the equity team, and the confidential address to reach them</t>
+          <t>Who is on the equity team, and their confidential email</t>
         </is>
       </c>
       <c r="D6" s="8" t="n"/>
@@ -591,7 +591,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Published by the equity team with input from the adjudication core and Org Comm</t>
+          <t>The equity team writes it, with input from the adjudication core and organising committee</t>
         </is>
       </c>
       <c r="E7" s="10" t="n"/>
@@ -609,12 +609,12 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Photos of Shivangi Sharma and Garvit Gosain</t>
+          <t>A photo of Garvit Gosain</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>They are on the site with their initials until then</t>
+          <t>The card shows initials until then</t>
         </is>
       </c>
       <c r="E8" s="10" t="n"/>

</xml_diff>